<commit_message>
Stabilize pre-import access and align import templates
Part 1 — units RLS (source-only migration, NOT applied):
the legacy "Units viewable by everyone" policy has no TO clause, so anon
could read unit titles (verified live). Drop it and replace with an
authenticated-only policy scoped by can_access_subject, matching the
content-gate model; content staff keep the FOR ALL manage policy.
6 static security tests incl. a guard against re-opening PUBLIC access.

Part 2 — import templates aligned with subject grouping:
dry-run now warns (non-blocking) on non-unified separators, the
non-approved «الإسلامية - ...» spelling, and mismatched parent spellings
of the same family — reusing the subject-grouping helpers. Template 01
regenerated with a grouped example row and naming instructions; README
documents the convention. 6 new dry-run tests.

No DML, no data changes, no schema changes, no import, no
payment/auth/storage changes.
</commit_message>
<xml_diff>
--- a/docs/content-templates/01_subjects_template.xlsx
+++ b/docs/content-templates/01_subjects_template.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="50">
   <si>
     <t>01 — نموذج المواد الدراسية</t>
   </si>
@@ -41,7 +41,7 @@
     <t>name *</t>
   </si>
   <si>
-    <t>مثال: الفيزياء</t>
+    <t>ملاحظة: مادة عادية: «الفيزياء» — مادة مقسّمة: «المادة الكبرى - القسم» — مثال: التربية الإسلامية - السيرة النبوية</t>
   </si>
   <si>
     <t>grade_slug *</t>
@@ -116,6 +116,18 @@
     <t>ابدأ بتحديد grade_slug و track_code قبل تعبئة المواد.</t>
   </si>
   <si>
+    <t>تقسيم المواد: الاسم بصيغة «اسم المادة الكبرى - اسم القسم الفرعي» والفاصل مسافة + شرطة + مسافة (" - ") حرفياً.</t>
+  </si>
+  <si>
+    <t>المعتمد دائماً «التربية الإسلامية - ...» — لا تستخدم «الإسلامية - ...».</t>
+  </si>
+  <si>
+    <t>وحّد هجاء اسم المادة الكبرى عبر كل أقسامها وإلا ظهرت كمواد منفصلة للطالب.</t>
+  </si>
+  <si>
+    <t>القيم المعتمدة للصف الأول: docs/SUBJECT-GROUPING-GRADE-10-YEMEN-CONTENT-GUIDE.md</t>
+  </si>
+  <si>
     <t>phys-g10-aden</t>
   </si>
   <si>
@@ -138,6 +150,18 @@
   </si>
   <si>
     <t>مسودة</t>
+  </si>
+  <si>
+    <t>islam-g10-sira</t>
+  </si>
+  <si>
+    <t>التربية الإسلامية - السيرة النبوية</t>
+  </si>
+  <si>
+    <t>BookOpen</t>
+  </si>
+  <si>
+    <t>#27ae60</t>
   </si>
 </sst>
 </file>
@@ -535,7 +559,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -701,6 +725,38 @@
         <v>33</v>
       </c>
     </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>27</v>
+      </c>
+      <c r="B24" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>27</v>
+      </c>
+      <c r="B25" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>27</v>
+      </c>
+      <c r="B26" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>27</v>
+      </c>
+      <c r="B27" t="s">
+        <v>37</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -709,7 +765,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -752,34 +808,66 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="B2" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="C2" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="D2" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="E2">
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="G2" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="H2">
+        <v>9</v>
+      </c>
+      <c r="I2" t="s">
+        <v>44</v>
+      </c>
+      <c r="J2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D3" t="s">
+        <v>44</v>
+      </c>
+      <c r="E3">
         <v>1</v>
       </c>
-      <c r="I2" t="s">
-        <v>40</v>
-      </c>
-      <c r="J2" t="s">
-        <v>41</v>
+      <c r="F3" t="s">
+        <v>48</v>
+      </c>
+      <c r="G3" t="s">
+        <v>49</v>
+      </c>
+      <c r="H3">
+        <v>2</v>
+      </c>
+      <c r="I3" t="s">
+        <v>44</v>
+      </c>
+      <c r="J3" t="s">
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>